<commit_message>
Tarife: Date actuale actualizate după setarea vara-toamna-2026 și iarna-2026 pe platforme (prețurile site-ului neschimbate)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uY5nf9QuxxsdiVUBPotuB
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="260">
   <si>
     <t xml:space="preserve">Strategia de prețuri – Travel Concept - Silver Mountain (A13)</t>
   </si>
@@ -817,7 +817,7 @@
     <t xml:space="preserve">Ultima zi cu tarif pe site</t>
   </si>
   <si>
-    <t xml:space="preserve">Date actuale – citite din conturi pe 21.10.2026</t>
+    <t xml:space="preserve">Date actuale – setate și verificate live în conturi pe 21.10.2026, ora 17:30</t>
   </si>
   <si>
     <t xml:space="preserve">Instantaneu pentru comparație. Actualizează-l când verifici din nou platformele.</t>
@@ -838,15 +838,18 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">21.10 – 30.11.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Airbnb/Travelminit cu 64% peste site/Booking</t>
+    <t xml:space="preserve">22.10 – 30.11.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setat 21.10.2026 conform tabelului (înainte: Booking 900, Airbnb 1.480, Travelminit 1.480). Site 900. Ocupat: 28.10–03.11, 28–29.11.</t>
   </si>
   <si>
     <t xml:space="preserve">01.12 – 20.12.2026</t>
   </si>
   <si>
+    <t xml:space="preserve">Setat 21.10.2026 conform tabelului (înainte 1.300 peste tot). Site 1.250.</t>
+  </si>
+  <si>
     <t xml:space="preserve">21.12 – 27.12.2026</t>
   </si>
   <si>
@@ -883,7 +886,7 @@
     <t xml:space="preserve">Booking: Standard Rate nerambursabil; planuri derivate 2–7 zile (-10% … -33%), flexibile 14 zile; plan „Sarbatori – Nerambursabil”; Mobile rate 10% activ din 07.06.2026; Genius neactiv.</t>
   </si>
   <si>
-    <t xml:space="preserve">Airbnb: preț de bază 1.480 lei → câștigi 1.251 lei (taxă unică gazdă ≈15,5%); reducere săptămânală 32%, lunară 33%; sejur 2–30 nopți; tarifare inteligentă oprită; sugestia Airbnb: 531 lei.</t>
+    <t xml:space="preserve">Airbnb: (verificat la 1.480 lei → câștigi 1.251 lei (taxă unică gazdă ≈15,5%)); reducerile 2–6 nopți șterse, rămân săptămânală 32%, lunară 33%; sejur 2–30 nopți; tarifare inteligentă oprită; sugestia Airbnb: 531 lei.</t>
   </si>
   <si>
     <t xml:space="preserve">Travelminit: nivel de comision net 12%; poziția 41 în Poiana Brașov (apartamente); reducere pe mobil afișată ca activă; nopți minime nesetate (Automatic); politică „sarbatori” cu avans.</t>
@@ -1864,41 +1867,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L1" s="2"/>
       <c r="M1" s="50" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5157,15 +5160,15 @@
       </c>
       <c r="L5" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$6="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A5,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>900</v>
+        <v>1130</v>
       </c>
       <c r="M5" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$6="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A5,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1480</v>
+        <v>920</v>
       </c>
       <c r="N5" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$6="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A5,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1480</v>
+        <v>980</v>
       </c>
       <c r="O5" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$6="","",Sezoane!M6)</f>
@@ -5243,15 +5246,15 @@
       </c>
       <c r="L6" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$7="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A6,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1300</v>
+        <v>1580</v>
       </c>
       <c r="M6" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$7="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A6,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1300</v>
+        <v>1420</v>
       </c>
       <c r="N6" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$7="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A6,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1300</v>
+        <v>1360</v>
       </c>
       <c r="O6" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$7="","",Sezoane!M7)</f>
@@ -25062,13 +25065,13 @@
         <v>229</v>
       </c>
       <c r="C6" s="48" t="n">
-        <v>900</v>
+        <v>1130</v>
       </c>
       <c r="D6" s="48" t="n">
-        <v>1480</v>
+        <v>920</v>
       </c>
       <c r="E6" s="48" t="n">
-        <v>1480</v>
+        <v>980</v>
       </c>
       <c r="F6" s="38" t="s">
         <v>230</v>
@@ -25082,22 +25085,24 @@
         <v>231</v>
       </c>
       <c r="C7" s="48" t="n">
-        <v>1300</v>
+        <v>1580</v>
       </c>
       <c r="D7" s="48" t="n">
-        <v>1300</v>
+        <v>1420</v>
       </c>
       <c r="E7" s="48" t="n">
-        <v>1300</v>
-      </c>
-      <c r="F7" s="38"/>
+        <v>1360</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
         <v>65</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C8" s="48" t="n">
         <v>1500</v>
@@ -25115,7 +25120,7 @@
         <v>68</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C9" s="48" t="n">
         <v>1800</v>
@@ -25133,7 +25138,7 @@
         <v>69</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C10" s="48" t="n">
         <v>1350</v>
@@ -25151,7 +25156,7 @@
         <v>70</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C11" s="48" t="n">
         <v>1450</v>
@@ -25163,15 +25168,15 @@
         <v>1500</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C12" s="48" t="n">
         <v>900</v>
@@ -25183,7 +25188,7 @@
         <v>1380</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25204,7 +25209,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -25214,7 +25219,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
@@ -25224,7 +25229,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
@@ -25234,7 +25239,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
@@ -25244,7 +25249,7 @@
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B19" s="49"/>
       <c r="C19" s="49"/>
@@ -25254,7 +25259,7 @@
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B20" s="49"/>
       <c r="C20" s="49"/>
@@ -25264,7 +25269,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B21" s="49"/>
       <c r="C21" s="49"/>

</xml_diff>

<commit_message>
Tarife: Date actuale – Crăciun setat pe platforme (Booking 1890, Travelminit 1630, min 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uY5nf9QuxxsdiVUBPotuB
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="261">
   <si>
     <t xml:space="preserve">Strategia de prețuri – Travel Concept - Silver Mountain (A13)</t>
   </si>
@@ -851,6 +851,9 @@
   </si>
   <si>
     <t xml:space="preserve">21.12 – 27.12.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setat 21.10.2026. Booking: doar planul „Sarbatori – Nerambursabil” deschis (1.890, min 3, Mobile rate 10% inclus în calcul); Airbnb min 3, politică „Fermă” (cea mai strictă disponibilă pe date), reducerea săptămânală 32% rămâne (risc acceptat); Travelminit min 3, politica „sarbatori”. Site 1.500, min 3, fără reduceri.</t>
   </si>
   <si>
     <t xml:space="preserve">28.12.2026 – 04.01.2027</t>
@@ -1867,41 +1870,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L1" s="2"/>
       <c r="M1" s="50" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5332,7 +5335,7 @@
       </c>
       <c r="L7" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$8="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A7,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1500</v>
+        <v>1890</v>
       </c>
       <c r="M7" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$8="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A7,'Date actuale'!$A$6:$A$40,0)),""))</f>
@@ -5340,7 +5343,7 @@
       </c>
       <c r="N7" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$8="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A7,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1700</v>
+        <v>1630</v>
       </c>
       <c r="O7" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$8="","",Sezoane!M8)</f>
@@ -25105,22 +25108,24 @@
         <v>233</v>
       </c>
       <c r="C8" s="48" t="n">
-        <v>1500</v>
+        <v>1890</v>
       </c>
       <c r="D8" s="48" t="n">
         <v>1700</v>
       </c>
       <c r="E8" s="48" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F8" s="38"/>
+        <v>1630</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
         <v>68</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C9" s="48" t="n">
         <v>1800</v>
@@ -25138,7 +25143,7 @@
         <v>69</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C10" s="48" t="n">
         <v>1350</v>
@@ -25156,7 +25161,7 @@
         <v>70</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C11" s="48" t="n">
         <v>1450</v>
@@ -25168,15 +25173,15 @@
         <v>1500</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C12" s="48" t="n">
         <v>900</v>
@@ -25188,7 +25193,7 @@
         <v>1380</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25209,7 +25214,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -25219,7 +25224,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
@@ -25229,7 +25234,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
@@ -25239,7 +25244,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
@@ -25249,7 +25254,7 @@
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B19" s="49"/>
       <c r="C19" s="49"/>
@@ -25259,7 +25264,7 @@
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B20" s="49"/>
       <c r="C20" s="49"/>
@@ -25269,7 +25274,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B21" s="49"/>
       <c r="C21" s="49"/>

</xml_diff>

<commit_message>
Tarife: Revelion setat pe platforme (Booking 2270, Airbnb 2040, Travelminit 1960, min 4); Date actuale actualizate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uY5nf9QuxxsdiVUBPotuB
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="262">
   <si>
     <t xml:space="preserve">Strategia de prețuri – Travel Concept - Silver Mountain (A13)</t>
   </si>
@@ -857,6 +857,9 @@
   </si>
   <si>
     <t xml:space="preserve">28.12.2026 – 04.01.2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setat 21.10.2026 (înainte: Booking 1.800, Airbnb 2.000/min 5, Travelminit 2.000). Booking: doar „Sarbatori – Nerambursabil” 2.270, min 4 (Mobile rate inclus în calcul); Airbnb 2.040, min 4, „Fermă”, reducerea săptămânală 32% rămâne (risc acceptat); Travelminit 1.960, min 4, politica „sarbatori”. Site 1.800, min 4, fără reduceri.</t>
   </si>
   <si>
     <t xml:space="preserve">05.01 – 14.02.2027</t>
@@ -1870,41 +1873,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="L1" s="2"/>
       <c r="M1" s="50" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5421,15 +5424,15 @@
       </c>
       <c r="L8" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$9="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A8,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1800</v>
+        <v>2270</v>
       </c>
       <c r="M8" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$9="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A8,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>2000</v>
+        <v>2040</v>
       </c>
       <c r="N8" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$9="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A8,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>2000</v>
+        <v>1960</v>
       </c>
       <c r="O8" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$9="","",Sezoane!M9)</f>
@@ -25128,22 +25131,24 @@
         <v>235</v>
       </c>
       <c r="C9" s="48" t="n">
-        <v>1800</v>
+        <v>2270</v>
       </c>
       <c r="D9" s="48" t="n">
-        <v>2000</v>
+        <v>2040</v>
       </c>
       <c r="E9" s="48" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F9" s="38"/>
+        <v>1960</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
         <v>69</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C10" s="48" t="n">
         <v>1350</v>
@@ -25161,7 +25166,7 @@
         <v>70</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C11" s="48" t="n">
         <v>1450</v>
@@ -25173,15 +25178,15 @@
         <v>1500</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C12" s="48" t="n">
         <v>900</v>
@@ -25193,7 +25198,7 @@
         <v>1380</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25214,7 +25219,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -25224,7 +25229,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
@@ -25234,7 +25239,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
@@ -25244,7 +25249,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
@@ -25254,7 +25259,7 @@
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B19" s="49"/>
       <c r="C19" s="49"/>
@@ -25264,7 +25269,7 @@
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B20" s="49"/>
       <c r="C20" s="49"/>
@@ -25274,7 +25279,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B21" s="49"/>
       <c r="C21" s="49"/>

</xml_diff>

<commit_message>
Tarife: iarna-2027 și vacanța de schi setate pe platforme; Date actuale + anomalie după 07.03
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uY5nf9QuxxsdiVUBPotuB
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="263">
   <si>
     <t xml:space="preserve">Strategia de prețuri – Travel Concept - Silver Mountain (A13)</t>
   </si>
@@ -865,10 +865,13 @@
     <t xml:space="preserve">05.01 – 14.02.2027</t>
   </si>
   <si>
+    <t xml:space="preserve">Setat 21.10.2026 (înainte: Booking 1.350, Airbnb 1.450, Travelminit 1.450). Min 2 peste tot; Booking planuri 2–7 nopți −10…−33% (flexibile 14 zile). Site 1.350.</t>
+  </si>
+  <si>
     <t xml:space="preserve">15.02 – 07.03.2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Airbnb are 1.500 doar până la 28.02; din 01.03 – 900</t>
+    <t xml:space="preserve">Setat 21.10.2026 (înainte: Booking 1.450, Airbnb 1.500 / 900 din 01.03, Travelminit 1.500). 20–21.02 ocupat (rezervare existentă, neatins). Site 1.450.</t>
   </si>
   <si>
     <t xml:space="preserve">(fără sezon pe site)</t>
@@ -877,7 +880,7 @@
     <t xml:space="preserve">08.03 – 30.04.2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Site blocat; Airbnb 900 din 01.03; Travelminit 1.380</t>
+    <t xml:space="preserve">ANOMALIE de decis: site blocat (fără sezon), Booking/Airbnb 900, Travelminit 1.380; Travelminit fără reguli (min nopți/politică) din 08.03.</t>
   </si>
   <si>
     <t xml:space="preserve">Comisioane și setări observate</t>
@@ -1873,41 +1876,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L1" s="2"/>
       <c r="M1" s="50" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5510,15 +5513,15 @@
       </c>
       <c r="L9" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$10="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A9,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1350</v>
+        <v>1700</v>
       </c>
       <c r="M9" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$10="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A9,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1450</v>
+        <v>1530</v>
       </c>
       <c r="N9" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$10="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A9,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1450</v>
+        <v>1470</v>
       </c>
       <c r="O9" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$10="","",Sezoane!M10)</f>
@@ -5596,15 +5599,15 @@
       </c>
       <c r="L10" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$11="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A10,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1450</v>
+        <v>1830</v>
       </c>
       <c r="M10" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$11="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A10,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1500</v>
+        <v>1640</v>
       </c>
       <c r="N10" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$11="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A10,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1500</v>
+        <v>1580</v>
       </c>
       <c r="O10" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$11="","",Sezoane!M11)</f>
@@ -25151,42 +25154,44 @@
         <v>237</v>
       </c>
       <c r="C10" s="48" t="n">
-        <v>1350</v>
+        <v>1700</v>
       </c>
       <c r="D10" s="48" t="n">
-        <v>1450</v>
+        <v>1530</v>
       </c>
       <c r="E10" s="48" t="n">
-        <v>1450</v>
-      </c>
-      <c r="F10" s="38"/>
+        <v>1470</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
         <v>70</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C11" s="48" t="n">
-        <v>1450</v>
+        <v>1830</v>
       </c>
       <c r="D11" s="48" t="n">
-        <v>1500</v>
+        <v>1640</v>
       </c>
       <c r="E11" s="48" t="n">
-        <v>1500</v>
+        <v>1580</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C12" s="48" t="n">
         <v>900</v>
@@ -25198,7 +25203,7 @@
         <v>1380</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25219,7 +25224,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -25229,7 +25234,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B16" s="49"/>
       <c r="C16" s="49"/>
@@ -25239,7 +25244,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B17" s="49"/>
       <c r="C17" s="49"/>
@@ -25249,7 +25254,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
@@ -25259,7 +25264,7 @@
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B19" s="49"/>
       <c r="C19" s="49"/>
@@ -25269,7 +25274,7 @@
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B20" s="49"/>
       <c r="C20" s="49"/>
@@ -25279,7 +25284,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B21" s="49"/>
       <c r="C21" s="49"/>

</xml_diff>

<commit_message>
Tarife: primavara-2027 setat pe platforme; Date actuale actualizate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uY5nf9QuxxsdiVUBPotuB
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -883,7 +883,7 @@
     <t xml:space="preserve">08.03 – 30.06.2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Înainte de setare (21.10.2026): site blocat (fără sezon), Booking/Airbnb 900, Travelminit 1.380, Travelminit fără reguli din 08.03.</t>
+    <t xml:space="preserve">Setat 21.10.2026 (înainte: site blocat, Booking/Airbnb 900, Travelminit 1.380 fără reguli). Iunie deschis pe Booking (era închis din 01.06 și bloca prin iCal Airbnb/Travelminit/site). Travelminit: min 2, politică standard. Site 900.</t>
   </si>
   <si>
     <t xml:space="preserve">Comisioane și setări observate</t>
@@ -5714,15 +5714,15 @@
       </c>
       <c r="L11" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$12="","",IFERROR(INDEX('Date actuale'!$C$6:$C$40,MATCH(A11,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>900</v>
+        <v>1130</v>
       </c>
       <c r="M11" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$12="","",IFERROR(INDEX('Date actuale'!$D$6:$D$40,MATCH(A11,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>900</v>
+        <v>1020</v>
       </c>
       <c r="N11" s="32" t="n">
         <f aca="false">IF(Sezoane!$A$12="","",IFERROR(INDEX('Date actuale'!$E$6:$E$40,MATCH(A11,'Date actuale'!$A$6:$A$40,0)),""))</f>
-        <v>1380</v>
+        <v>980</v>
       </c>
       <c r="O11" s="25" t="str">
         <f aca="false">IF(Sezoane!$A$12="","",Sezoane!M12)</f>
@@ -25223,13 +25223,13 @@
         <v>243</v>
       </c>
       <c r="C12" s="48" t="n">
-        <v>900</v>
+        <v>1130</v>
       </c>
       <c r="D12" s="48" t="n">
-        <v>900</v>
+        <v>1020</v>
       </c>
       <c r="E12" s="48" t="n">
-        <v>1380</v>
+        <v>980</v>
       </c>
       <c r="F12" s="38" t="s">
         <v>244</v>

</xml_diff>

<commit_message>
Pages: _config.yml exclude documentatia interna, tarife.xlsx, apps-script si scripturile de build; tarife.xlsx fara numere de rezervare; CLAUDE.md actualizat (audit 2026-10-21)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pricing/tarife.xlsx
+++ b/pricing/tarife.xlsx
@@ -399,7 +399,7 @@
     <t xml:space="preserve">Comision platformă</t>
   </si>
   <si>
-    <t xml:space="preserve">Booking 15% (din rezervările 6131205469, 5429915812, 6470558532). Airbnb: taxă unică gazdă 15,5% (editor Airbnb: 1.480 lei → câștigi 1.251 lei). Travelminit: „Nivelul de comisionare actual 12%” (admin → Îmbunătățirea poziției).</t>
+    <t xml:space="preserve">Booking 15% (din 3 rezervări Booking reale). Airbnb: taxă unică gazdă 15,5% (editor Airbnb: 1.480 lei → câștigi 1.251 lei). Travelminit: „Nivelul de comisionare actual 12%” (admin → Îmbunătățirea poziției).</t>
   </si>
   <si>
     <t xml:space="preserve">Costuri procesare plată</t>
@@ -889,10 +889,10 @@
     <t xml:space="preserve">Comisioane și setări observate</t>
   </si>
   <si>
-    <t xml:space="preserve">Booking: rez. 6131205469 – suma comisionabilă 3.633 lei, comision și costuri 596,55 lei (16,4%); total oaspete 3.969 lei (taxe locale 336 lei incluse, scăzute din baza de comision).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Booking: rez. 5429915812 – 1.362 lei comisionabil, 223,25 lei comision (16,4%); rez. 6470558532 – 2.253 lei, 368,49 lei (16,4%).</t>
+    <t xml:space="preserve">Booking, rezervarea 1 – suma comisionabilă 3.633 lei, comision și costuri 596,55 lei (16,4%); total oaspete 3.969 lei (taxe locale 336 lei incluse, scăzute din baza de comision).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking, rezervarea 2 – 1.362 lei comisionabil, 223,25 lei comision (16,4%); rezervarea 3 – 2.253 lei, 368,49 lei (16,4%).</t>
   </si>
   <si>
     <t xml:space="preserve">Booking: Standard Rate nerambursabil; planuri derivate 2–7 zile (-10% … -33%), flexibile 14 zile; plan „Sarbatori – Nerambursabil”; Mobile rate 10% activ din 07.06.2026; Genius neactiv.</t>

</xml_diff>